<commit_message>
Moved to manifest pipeline
</commit_message>
<xml_diff>
--- a/outputs/run_manifest.xlsx
+++ b/outputs/run_manifest.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL25"/>
+  <dimension ref="A1:CQ25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,140 +742,165 @@
       </c>
       <c r="BK1" s="1" t="inlineStr">
         <is>
+          <t>perturbation_stage_logging</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>perturbation_progress_logging</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
           <t>perturbation_sample_count</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>perturbation_candidate_units</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>perturbation_target_units</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>perturbation_trust_trials</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>perturbation_progress_sample_interval</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>perturbation_random_strength</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>explainability_method</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>explainability_target</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>service_source</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>model_role</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>fit_decision</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BX1" s="1" t="inlineStr">
         <is>
           <t>fit_reason</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BY1" s="1" t="inlineStr">
         <is>
           <t>realism_score</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="BZ1" s="1" t="inlineStr">
         <is>
           <t>domain_alignment</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="CA1" s="1" t="inlineStr">
         <is>
           <t>dataset_hint</t>
         </is>
       </c>
-      <c r="BW1" s="1" t="inlineStr">
+      <c r="CB1" s="1" t="inlineStr">
         <is>
           <t>hf_pipeline_tag</t>
         </is>
       </c>
-      <c r="BX1" s="1" t="inlineStr">
+      <c r="CC1" s="1" t="inlineStr">
         <is>
           <t>hf_downloads</t>
         </is>
       </c>
-      <c r="BY1" s="1" t="inlineStr">
+      <c r="CD1" s="1" t="inlineStr">
         <is>
           <t>hf_likes</t>
         </is>
       </c>
-      <c r="BZ1" s="1" t="inlineStr">
+      <c r="CE1" s="1" t="inlineStr">
         <is>
           <t>hf_dataset_id</t>
         </is>
       </c>
-      <c r="CA1" s="1" t="inlineStr">
+      <c r="CF1" s="1" t="inlineStr">
         <is>
           <t>downloads</t>
         </is>
       </c>
-      <c r="CB1" s="1" t="inlineStr">
+      <c r="CG1" s="1" t="inlineStr">
         <is>
           <t>likes</t>
         </is>
       </c>
-      <c r="CC1" s="1" t="inlineStr">
+      <c r="CH1" s="1" t="inlineStr">
         <is>
           <t>model_size</t>
         </is>
       </c>
-      <c r="CD1" s="1" t="inlineStr">
+      <c r="CI1" s="1" t="inlineStr">
         <is>
           <t>params_count</t>
         </is>
       </c>
-      <c r="CE1" s="1" t="inlineStr">
+      <c r="CJ1" s="1" t="inlineStr">
         <is>
           <t>pipeline_tag</t>
         </is>
       </c>
-      <c r="CF1" s="1" t="inlineStr">
+      <c r="CK1" s="1" t="inlineStr">
         <is>
           <t>library_name</t>
         </is>
       </c>
-      <c r="CG1" s="1" t="inlineStr">
+      <c r="CL1" s="1" t="inlineStr">
         <is>
           <t>license</t>
         </is>
       </c>
-      <c r="CH1" s="1" t="inlineStr">
+      <c r="CM1" s="1" t="inlineStr">
         <is>
           <t>tags</t>
         </is>
       </c>
-      <c r="CI1" s="1" t="inlineStr">
+      <c r="CN1" s="1" t="inlineStr">
         <is>
           <t>last_modified</t>
         </is>
       </c>
-      <c r="CJ1" s="1" t="inlineStr">
+      <c r="CO1" s="1" t="inlineStr">
         <is>
           <t>hf_author</t>
         </is>
       </c>
-      <c r="CK1" s="1" t="inlineStr">
+      <c r="CP1" s="1" t="inlineStr">
         <is>
           <t>hf_url</t>
         </is>
       </c>
-      <c r="CL1" s="1" t="inlineStr">
+      <c r="CQ1" s="1" t="inlineStr">
         <is>
           <t>hf_service_meta_json</t>
         </is>
@@ -979,7 +1004,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -1070,58 +1095,68 @@
       <c r="BJ2" t="b">
         <v>1</v>
       </c>
-      <c r="BK2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL2" t="n">
+      <c r="BK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN2" t="n">
         <v>4</v>
       </c>
-      <c r="BM2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN2" t="inlineStr">
+      <c r="BO2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS2" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO2" t="inlineStr">
+      <c r="BT2" t="inlineStr">
         <is>
           <t>class_label</t>
         </is>
       </c>
-      <c r="BP2" t="inlineStr">
+      <c r="BU2" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ2" t="inlineStr">
+      <c r="BV2" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR2" t="inlineStr">
+      <c r="BW2" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS2" t="inlineStr">
+      <c r="BX2" t="inlineStr">
         <is>
           <t>registry-compatible task=text_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr"/>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>text-classification</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
       <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>text-classification</t>
+        </is>
+      </c>
       <c r="CC2" t="inlineStr"/>
       <c r="CD2" t="inlineStr"/>
       <c r="CE2" t="inlineStr"/>
@@ -1131,7 +1166,12 @@
       <c r="CI2" t="inlineStr"/>
       <c r="CJ2" t="inlineStr"/>
       <c r="CK2" t="inlineStr"/>
-      <c r="CL2" t="inlineStr">
+      <c r="CL2" t="inlineStr"/>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "rotten_tomatoes", "dataset_variant": 0, "knob_variant": 0, "model_family": "tinybert", "model_registry_key": "tinybert-general-4l_textcls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -1239,7 +1279,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -1330,58 +1370,68 @@
       <c r="BJ3" t="b">
         <v>1</v>
       </c>
-      <c r="BK3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL3" t="n">
+      <c r="BK3" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL3" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN3" t="n">
         <v>4</v>
       </c>
-      <c r="BM3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN3" t="inlineStr">
+      <c r="BO3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS3" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO3" t="inlineStr">
+      <c r="BT3" t="inlineStr">
         <is>
           <t>class_label</t>
         </is>
       </c>
-      <c r="BP3" t="inlineStr">
+      <c r="BU3" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ3" t="inlineStr">
+      <c r="BV3" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR3" t="inlineStr">
+      <c r="BW3" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS3" t="inlineStr">
+      <c r="BX3" t="inlineStr">
         <is>
           <t>registry-compatible task=text_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr"/>
-      <c r="BW3" t="inlineStr">
-        <is>
-          <t>text-classification</t>
-        </is>
-      </c>
-      <c r="BX3" t="inlineStr"/>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
       <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>text-classification</t>
+        </is>
+      </c>
       <c r="CC3" t="inlineStr"/>
       <c r="CD3" t="inlineStr"/>
       <c r="CE3" t="inlineStr"/>
@@ -1391,7 +1441,12 @@
       <c r="CI3" t="inlineStr"/>
       <c r="CJ3" t="inlineStr"/>
       <c r="CK3" t="inlineStr"/>
-      <c r="CL3" t="inlineStr">
+      <c r="CL3" t="inlineStr"/>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "glue_cola", "dataset_variant": 0, "knob_variant": 0, "model_family": "albert", "model_registry_key": "albert-base-v2_textcls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -1499,7 +1554,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -1590,58 +1645,68 @@
       <c r="BJ4" t="b">
         <v>1</v>
       </c>
-      <c r="BK4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL4" t="n">
+      <c r="BK4" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL4" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN4" t="n">
         <v>4</v>
       </c>
-      <c r="BM4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN4" t="inlineStr">
+      <c r="BO4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS4" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO4" t="inlineStr">
+      <c r="BT4" t="inlineStr">
         <is>
           <t>token_label</t>
         </is>
       </c>
-      <c r="BP4" t="inlineStr">
+      <c r="BU4" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ4" t="inlineStr">
+      <c r="BV4" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR4" t="inlineStr">
+      <c r="BW4" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS4" t="inlineStr">
+      <c r="BX4" t="inlineStr">
         <is>
           <t>registry-compatible task=token_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr"/>
-      <c r="BW4" t="inlineStr">
-        <is>
-          <t>token-classification</t>
-        </is>
-      </c>
-      <c r="BX4" t="inlineStr"/>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
       <c r="CA4" t="inlineStr"/>
-      <c r="CB4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr">
+        <is>
+          <t>token-classification</t>
+        </is>
+      </c>
       <c r="CC4" t="inlineStr"/>
       <c r="CD4" t="inlineStr"/>
       <c r="CE4" t="inlineStr"/>
@@ -1651,7 +1716,12 @@
       <c r="CI4" t="inlineStr"/>
       <c r="CJ4" t="inlineStr"/>
       <c r="CK4" t="inlineStr"/>
-      <c r="CL4" t="inlineStr">
+      <c r="CL4" t="inlineStr"/>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "conllpp", "dataset_variant": 0, "knob_variant": 0, "model_family": "roberta", "model_registry_key": "roberta-base_tokencls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -1759,7 +1829,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1850,58 +1920,68 @@
       <c r="BJ5" t="b">
         <v>1</v>
       </c>
-      <c r="BK5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL5" t="n">
+      <c r="BK5" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL5" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN5" t="n">
         <v>4</v>
       </c>
-      <c r="BM5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN5" t="inlineStr">
+      <c r="BO5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS5" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO5" t="inlineStr">
+      <c r="BT5" t="inlineStr">
         <is>
           <t>token_label</t>
         </is>
       </c>
-      <c r="BP5" t="inlineStr">
+      <c r="BU5" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ5" t="inlineStr">
+      <c r="BV5" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR5" t="inlineStr">
+      <c r="BW5" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS5" t="inlineStr">
+      <c r="BX5" t="inlineStr">
         <is>
           <t>registry-compatible task=token_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT5" t="inlineStr"/>
-      <c r="BU5" t="inlineStr"/>
-      <c r="BV5" t="inlineStr"/>
-      <c r="BW5" t="inlineStr">
-        <is>
-          <t>token-classification</t>
-        </is>
-      </c>
-      <c r="BX5" t="inlineStr"/>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
       <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr">
+        <is>
+          <t>token-classification</t>
+        </is>
+      </c>
       <c r="CC5" t="inlineStr"/>
       <c r="CD5" t="inlineStr"/>
       <c r="CE5" t="inlineStr"/>
@@ -1911,7 +1991,12 @@
       <c r="CI5" t="inlineStr"/>
       <c r="CJ5" t="inlineStr"/>
       <c r="CK5" t="inlineStr"/>
-      <c r="CL5" t="inlineStr">
+      <c r="CL5" t="inlineStr"/>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="inlineStr"/>
+      <c r="CP5" t="inlineStr"/>
+      <c r="CQ5" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "conllpp", "dataset_variant": 0, "knob_variant": 0, "model_family": "mobilebert", "model_registry_key": "mobilebert-uncased_tokencls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -2019,7 +2104,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -2110,58 +2195,68 @@
       <c r="BJ6" t="b">
         <v>1</v>
       </c>
-      <c r="BK6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL6" t="n">
+      <c r="BK6" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL6" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN6" t="n">
         <v>4</v>
       </c>
-      <c r="BM6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN6" t="inlineStr">
+      <c r="BO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS6" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO6" t="inlineStr">
+      <c r="BT6" t="inlineStr">
         <is>
           <t>similarity_score</t>
         </is>
       </c>
-      <c r="BP6" t="inlineStr">
+      <c r="BU6" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ6" t="inlineStr">
+      <c r="BV6" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR6" t="inlineStr">
+      <c r="BW6" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS6" t="inlineStr">
+      <c r="BX6" t="inlineStr">
         <is>
           <t>registry-compatible task=sentence_similarity training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
-      <c r="BV6" t="inlineStr"/>
-      <c r="BW6" t="inlineStr">
-        <is>
-          <t>sentence-similarity</t>
-        </is>
-      </c>
-      <c r="BX6" t="inlineStr"/>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
       <c r="CA6" t="inlineStr"/>
-      <c r="CB6" t="inlineStr"/>
+      <c r="CB6" t="inlineStr">
+        <is>
+          <t>sentence-similarity</t>
+        </is>
+      </c>
       <c r="CC6" t="inlineStr"/>
       <c r="CD6" t="inlineStr"/>
       <c r="CE6" t="inlineStr"/>
@@ -2171,7 +2266,12 @@
       <c r="CI6" t="inlineStr"/>
       <c r="CJ6" t="inlineStr"/>
       <c r="CK6" t="inlineStr"/>
-      <c r="CL6" t="inlineStr">
+      <c r="CL6" t="inlineStr"/>
+      <c r="CM6" t="inlineStr"/>
+      <c r="CN6" t="inlineStr"/>
+      <c r="CO6" t="inlineStr"/>
+      <c r="CP6" t="inlineStr"/>
+      <c r="CQ6" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "glue_stsb", "dataset_variant": 0, "knob_variant": 0, "model_family": "tinybert", "model_registry_key": "tinybert-general-4l_similarity", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -2279,7 +2379,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 5e-05, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 5e-05, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -2370,58 +2470,68 @@
       <c r="BJ7" t="b">
         <v>1</v>
       </c>
-      <c r="BK7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL7" t="n">
+      <c r="BK7" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN7" t="n">
         <v>4</v>
       </c>
-      <c r="BM7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN7" t="inlineStr">
+      <c r="BO7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS7" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO7" t="inlineStr">
+      <c r="BT7" t="inlineStr">
         <is>
           <t>similarity_score</t>
         </is>
       </c>
-      <c r="BP7" t="inlineStr">
+      <c r="BU7" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ7" t="inlineStr">
+      <c r="BV7" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR7" t="inlineStr">
+      <c r="BW7" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS7" t="inlineStr">
+      <c r="BX7" t="inlineStr">
         <is>
           <t>registry-compatible task=sentence_similarity training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT7" t="inlineStr"/>
-      <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
-      <c r="BW7" t="inlineStr">
-        <is>
-          <t>sentence-similarity</t>
-        </is>
-      </c>
-      <c r="BX7" t="inlineStr"/>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
       <c r="CA7" t="inlineStr"/>
-      <c r="CB7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr">
+        <is>
+          <t>sentence-similarity</t>
+        </is>
+      </c>
       <c r="CC7" t="inlineStr"/>
       <c r="CD7" t="inlineStr"/>
       <c r="CE7" t="inlineStr"/>
@@ -2431,7 +2541,12 @@
       <c r="CI7" t="inlineStr"/>
       <c r="CJ7" t="inlineStr"/>
       <c r="CK7" t="inlineStr"/>
-      <c r="CL7" t="inlineStr">
+      <c r="CL7" t="inlineStr"/>
+      <c r="CM7" t="inlineStr"/>
+      <c r="CN7" t="inlineStr"/>
+      <c r="CO7" t="inlineStr"/>
+      <c r="CP7" t="inlineStr"/>
+      <c r="CQ7" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "glue_rte_similarity", "dataset_variant": 0, "knob_variant": 0, "model_family": "bert", "model_registry_key": "bert-base-uncased_similarity", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -2535,7 +2650,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -2626,58 +2741,68 @@
       <c r="BJ8" t="b">
         <v>1</v>
       </c>
-      <c r="BK8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL8" t="n">
+      <c r="BK8" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL8" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN8" t="n">
         <v>4</v>
       </c>
-      <c r="BM8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN8" t="inlineStr">
+      <c r="BO8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS8" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO8" t="inlineStr">
+      <c r="BT8" t="inlineStr">
         <is>
           <t>masked_token</t>
         </is>
       </c>
-      <c r="BP8" t="inlineStr">
+      <c r="BU8" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ8" t="inlineStr">
+      <c r="BV8" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR8" t="inlineStr">
+      <c r="BW8" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS8" t="inlineStr">
+      <c r="BX8" t="inlineStr">
         <is>
           <t>registry-compatible task=fill_mask training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT8" t="inlineStr"/>
-      <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
-      <c r="BW8" t="inlineStr">
-        <is>
-          <t>fill-mask</t>
-        </is>
-      </c>
-      <c r="BX8" t="inlineStr"/>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
       <c r="CA8" t="inlineStr"/>
-      <c r="CB8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>fill-mask</t>
+        </is>
+      </c>
       <c r="CC8" t="inlineStr"/>
       <c r="CD8" t="inlineStr"/>
       <c r="CE8" t="inlineStr"/>
@@ -2687,7 +2812,12 @@
       <c r="CI8" t="inlineStr"/>
       <c r="CJ8" t="inlineStr"/>
       <c r="CK8" t="inlineStr"/>
-      <c r="CL8" t="inlineStr">
+      <c r="CL8" t="inlineStr"/>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
+      <c r="CQ8" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "tinystories_fillmask", "dataset_variant": 0, "knob_variant": 0, "model_family": "roberta", "model_registry_key": "distilroberta-base_fillmask", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -2795,7 +2925,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 128, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -2886,58 +3016,68 @@
       <c r="BJ9" t="b">
         <v>1</v>
       </c>
-      <c r="BK9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL9" t="n">
+      <c r="BK9" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL9" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN9" t="n">
         <v>4</v>
       </c>
-      <c r="BM9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN9" t="inlineStr">
+      <c r="BO9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS9" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO9" t="inlineStr">
+      <c r="BT9" t="inlineStr">
         <is>
           <t>masked_token</t>
         </is>
       </c>
-      <c r="BP9" t="inlineStr">
+      <c r="BU9" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ9" t="inlineStr">
+      <c r="BV9" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR9" t="inlineStr">
+      <c r="BW9" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS9" t="inlineStr">
+      <c r="BX9" t="inlineStr">
         <is>
           <t>registry-compatible task=fill_mask training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT9" t="inlineStr"/>
-      <c r="BU9" t="inlineStr"/>
-      <c r="BV9" t="inlineStr"/>
-      <c r="BW9" t="inlineStr">
-        <is>
-          <t>fill-mask</t>
-        </is>
-      </c>
-      <c r="BX9" t="inlineStr"/>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
       <c r="CA9" t="inlineStr"/>
-      <c r="CB9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr">
+        <is>
+          <t>fill-mask</t>
+        </is>
+      </c>
       <c r="CC9" t="inlineStr"/>
       <c r="CD9" t="inlineStr"/>
       <c r="CE9" t="inlineStr"/>
@@ -2947,7 +3087,12 @@
       <c r="CI9" t="inlineStr"/>
       <c r="CJ9" t="inlineStr"/>
       <c r="CK9" t="inlineStr"/>
-      <c r="CL9" t="inlineStr">
+      <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="inlineStr"/>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="inlineStr"/>
+      <c r="CP9" t="inlineStr"/>
+      <c r="CQ9" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "wikitext2", "dataset_variant": 0, "knob_variant": 0, "model_family": "electra", "model_registry_key": "electra-base-generator_fillmask", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -3055,7 +3200,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 192, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -3146,58 +3291,68 @@
       <c r="BJ10" t="b">
         <v>1</v>
       </c>
-      <c r="BK10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL10" t="n">
+      <c r="BK10" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL10" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN10" t="n">
         <v>4</v>
       </c>
-      <c r="BM10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN10" t="inlineStr">
+      <c r="BO10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS10" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO10" t="inlineStr">
+      <c r="BT10" t="inlineStr">
         <is>
           <t>generated_token</t>
         </is>
       </c>
-      <c r="BP10" t="inlineStr">
+      <c r="BU10" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ10" t="inlineStr">
+      <c r="BV10" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR10" t="inlineStr">
+      <c r="BW10" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS10" t="inlineStr">
+      <c r="BX10" t="inlineStr">
         <is>
           <t>registry-compatible task=text_generation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT10" t="inlineStr"/>
-      <c r="BU10" t="inlineStr"/>
-      <c r="BV10" t="inlineStr"/>
-      <c r="BW10" t="inlineStr">
-        <is>
-          <t>text-generation</t>
-        </is>
-      </c>
-      <c r="BX10" t="inlineStr"/>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
       <c r="CA10" t="inlineStr"/>
-      <c r="CB10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr">
+        <is>
+          <t>text-generation</t>
+        </is>
+      </c>
       <c r="CC10" t="inlineStr"/>
       <c r="CD10" t="inlineStr"/>
       <c r="CE10" t="inlineStr"/>
@@ -3207,7 +3362,12 @@
       <c r="CI10" t="inlineStr"/>
       <c r="CJ10" t="inlineStr"/>
       <c r="CK10" t="inlineStr"/>
-      <c r="CL10" t="inlineStr">
+      <c r="CL10" t="inlineStr"/>
+      <c r="CM10" t="inlineStr"/>
+      <c r="CN10" t="inlineStr"/>
+      <c r="CO10" t="inlineStr"/>
+      <c r="CP10" t="inlineStr"/>
+      <c r="CQ10" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "rotten_tomatoes_lm", "dataset_variant": 0, "knob_variant": 0, "model_family": "dialogpt", "model_registry_key": "dialogpt-small_textgen", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -3319,7 +3479,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -3410,58 +3570,68 @@
       <c r="BJ11" t="b">
         <v>1</v>
       </c>
-      <c r="BK11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL11" t="n">
+      <c r="BK11" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL11" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN11" t="n">
         <v>4</v>
       </c>
-      <c r="BM11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN11" t="inlineStr">
+      <c r="BO11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS11" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO11" t="inlineStr">
+      <c r="BT11" t="inlineStr">
         <is>
           <t>generated_token</t>
         </is>
       </c>
-      <c r="BP11" t="inlineStr">
+      <c r="BU11" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ11" t="inlineStr">
+      <c r="BV11" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR11" t="inlineStr">
+      <c r="BW11" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS11" t="inlineStr">
+      <c r="BX11" t="inlineStr">
         <is>
           <t>registry-compatible task=text_generation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT11" t="inlineStr"/>
-      <c r="BU11" t="inlineStr"/>
-      <c r="BV11" t="inlineStr"/>
-      <c r="BW11" t="inlineStr">
-        <is>
-          <t>text-generation</t>
-        </is>
-      </c>
-      <c r="BX11" t="inlineStr"/>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
       <c r="CA11" t="inlineStr"/>
-      <c r="CB11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr">
+        <is>
+          <t>text-generation</t>
+        </is>
+      </c>
       <c r="CC11" t="inlineStr"/>
       <c r="CD11" t="inlineStr"/>
       <c r="CE11" t="inlineStr"/>
@@ -3471,7 +3641,12 @@
       <c r="CI11" t="inlineStr"/>
       <c r="CJ11" t="inlineStr"/>
       <c r="CK11" t="inlineStr"/>
-      <c r="CL11" t="inlineStr">
+      <c r="CL11" t="inlineStr"/>
+      <c r="CM11" t="inlineStr"/>
+      <c r="CN11" t="inlineStr"/>
+      <c r="CO11" t="inlineStr"/>
+      <c r="CP11" t="inlineStr"/>
+      <c r="CQ11" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "arxiv_summarization_lm", "dataset_variant": 0, "knob_variant": 0, "model_family": "opt", "model_registry_key": "opt-125m_textgen", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -3583,7 +3758,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
@@ -3674,58 +3849,68 @@
       <c r="BJ12" t="b">
         <v>1</v>
       </c>
-      <c r="BK12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL12" t="n">
+      <c r="BK12" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL12" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN12" t="n">
         <v>4</v>
       </c>
-      <c r="BM12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN12" t="inlineStr">
+      <c r="BO12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS12" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO12" t="inlineStr">
+      <c r="BT12" t="inlineStr">
         <is>
           <t>summary_token</t>
         </is>
       </c>
-      <c r="BP12" t="inlineStr">
+      <c r="BU12" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ12" t="inlineStr">
+      <c r="BV12" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR12" t="inlineStr">
+      <c r="BW12" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS12" t="inlineStr">
+      <c r="BX12" t="inlineStr">
         <is>
           <t>registry-compatible task=text2text_generation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT12" t="inlineStr"/>
-      <c r="BU12" t="inlineStr"/>
-      <c r="BV12" t="inlineStr"/>
-      <c r="BW12" t="inlineStr">
-        <is>
-          <t>text2text-generation</t>
-        </is>
-      </c>
-      <c r="BX12" t="inlineStr"/>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
       <c r="CA12" t="inlineStr"/>
-      <c r="CB12" t="inlineStr"/>
+      <c r="CB12" t="inlineStr">
+        <is>
+          <t>text2text-generation</t>
+        </is>
+      </c>
       <c r="CC12" t="inlineStr"/>
       <c r="CD12" t="inlineStr"/>
       <c r="CE12" t="inlineStr"/>
@@ -3735,7 +3920,12 @@
       <c r="CI12" t="inlineStr"/>
       <c r="CJ12" t="inlineStr"/>
       <c r="CK12" t="inlineStr"/>
-      <c r="CL12" t="inlineStr">
+      <c r="CL12" t="inlineStr"/>
+      <c r="CM12" t="inlineStr"/>
+      <c r="CN12" t="inlineStr"/>
+      <c r="CO12" t="inlineStr"/>
+      <c r="CP12" t="inlineStr"/>
+      <c r="CQ12" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "cnn_dailymail", "dataset_variant": 0, "knob_variant": 0, "model_family": "t5", "model_registry_key": "flan-t5-base_text2text", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -3847,7 +4037,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_length": 256, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
@@ -3938,58 +4128,68 @@
       <c r="BJ13" t="b">
         <v>1</v>
       </c>
-      <c r="BK13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL13" t="n">
+      <c r="BK13" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL13" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN13" t="n">
         <v>4</v>
       </c>
-      <c r="BM13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN13" t="inlineStr">
+      <c r="BO13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS13" t="inlineStr">
         <is>
           <t>integrated_gradients</t>
         </is>
       </c>
-      <c r="BO13" t="inlineStr">
+      <c r="BT13" t="inlineStr">
         <is>
           <t>summary_token</t>
         </is>
       </c>
-      <c r="BP13" t="inlineStr">
+      <c r="BU13" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ13" t="inlineStr">
+      <c r="BV13" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR13" t="inlineStr">
+      <c r="BW13" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS13" t="inlineStr">
+      <c r="BX13" t="inlineStr">
         <is>
           <t>registry-compatible task=text2text_generation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT13" t="inlineStr"/>
-      <c r="BU13" t="inlineStr"/>
-      <c r="BV13" t="inlineStr"/>
-      <c r="BW13" t="inlineStr">
-        <is>
-          <t>text2text-generation</t>
-        </is>
-      </c>
-      <c r="BX13" t="inlineStr"/>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
       <c r="CA13" t="inlineStr"/>
-      <c r="CB13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>text2text-generation</t>
+        </is>
+      </c>
       <c r="CC13" t="inlineStr"/>
       <c r="CD13" t="inlineStr"/>
       <c r="CE13" t="inlineStr"/>
@@ -3999,7 +4199,12 @@
       <c r="CI13" t="inlineStr"/>
       <c r="CJ13" t="inlineStr"/>
       <c r="CK13" t="inlineStr"/>
-      <c r="CL13" t="inlineStr">
+      <c r="CL13" t="inlineStr"/>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
+      <c r="CO13" t="inlineStr"/>
+      <c r="CP13" t="inlineStr"/>
+      <c r="CQ13" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "cnn_dailymail", "dataset_variant": 0, "knob_variant": 0, "model_family": "codet5", "model_registry_key": "codet5-small_text2text", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -4107,7 +4312,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -4196,50 +4401,60 @@
       <c r="BJ14" t="b">
         <v>1</v>
       </c>
-      <c r="BK14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL14" t="n">
+      <c r="BK14" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL14" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN14" t="n">
         <v>4</v>
       </c>
-      <c r="BM14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN14" t="inlineStr"/>
-      <c r="BO14" t="inlineStr"/>
-      <c r="BP14" t="inlineStr">
+      <c r="BO14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ14" t="inlineStr">
+      <c r="BV14" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR14" t="inlineStr">
+      <c r="BW14" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS14" t="inlineStr">
+      <c r="BX14" t="inlineStr">
         <is>
           <t>registry-compatible task=image_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT14" t="inlineStr"/>
-      <c r="BU14" t="inlineStr"/>
-      <c r="BV14" t="inlineStr"/>
-      <c r="BW14" t="inlineStr">
-        <is>
-          <t>image-classification</t>
-        </is>
-      </c>
-      <c r="BX14" t="inlineStr"/>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
       <c r="CA14" t="inlineStr"/>
-      <c r="CB14" t="inlineStr"/>
+      <c r="CB14" t="inlineStr">
+        <is>
+          <t>image-classification</t>
+        </is>
+      </c>
       <c r="CC14" t="inlineStr"/>
       <c r="CD14" t="inlineStr"/>
       <c r="CE14" t="inlineStr"/>
@@ -4249,7 +4464,12 @@
       <c r="CI14" t="inlineStr"/>
       <c r="CJ14" t="inlineStr"/>
       <c r="CK14" t="inlineStr"/>
-      <c r="CL14" t="inlineStr">
+      <c r="CL14" t="inlineStr"/>
+      <c r="CM14" t="inlineStr"/>
+      <c r="CN14" t="inlineStr"/>
+      <c r="CO14" t="inlineStr"/>
+      <c r="CP14" t="inlineStr"/>
+      <c r="CQ14" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "fashion_mnist", "dataset_variant": 0, "knob_variant": 0, "model_family": "deit", "model_registry_key": "deit-tiny-patch16-224_imgcls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -4357,7 +4577,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "learning_rate": 5e-05, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 5e-05, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -4446,50 +4666,60 @@
       <c r="BJ15" t="b">
         <v>1</v>
       </c>
-      <c r="BK15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL15" t="n">
+      <c r="BK15" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL15" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN15" t="n">
         <v>4</v>
       </c>
-      <c r="BM15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN15" t="inlineStr"/>
-      <c r="BO15" t="inlineStr"/>
-      <c r="BP15" t="inlineStr">
+      <c r="BO15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ15" t="inlineStr">
+      <c r="BV15" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR15" t="inlineStr">
+      <c r="BW15" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS15" t="inlineStr">
+      <c r="BX15" t="inlineStr">
         <is>
           <t>registry-compatible task=image_classification training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT15" t="inlineStr"/>
-      <c r="BU15" t="inlineStr"/>
-      <c r="BV15" t="inlineStr"/>
-      <c r="BW15" t="inlineStr">
-        <is>
-          <t>image-classification</t>
-        </is>
-      </c>
-      <c r="BX15" t="inlineStr"/>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
       <c r="CA15" t="inlineStr"/>
-      <c r="CB15" t="inlineStr"/>
+      <c r="CB15" t="inlineStr">
+        <is>
+          <t>image-classification</t>
+        </is>
+      </c>
       <c r="CC15" t="inlineStr"/>
       <c r="CD15" t="inlineStr"/>
       <c r="CE15" t="inlineStr"/>
@@ -4499,7 +4729,12 @@
       <c r="CI15" t="inlineStr"/>
       <c r="CJ15" t="inlineStr"/>
       <c r="CK15" t="inlineStr"/>
-      <c r="CL15" t="inlineStr">
+      <c r="CL15" t="inlineStr"/>
+      <c r="CM15" t="inlineStr"/>
+      <c r="CN15" t="inlineStr"/>
+      <c r="CO15" t="inlineStr"/>
+      <c r="CP15" t="inlineStr"/>
+      <c r="CQ15" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "fashion_mnist", "dataset_variant": 0, "knob_variant": 0, "model_family": "resnet", "model_registry_key": "resnet-50_imgcls", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -4607,7 +4842,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -4696,50 +4931,60 @@
       <c r="BJ16" t="b">
         <v>1</v>
       </c>
-      <c r="BK16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL16" t="n">
+      <c r="BK16" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL16" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN16" t="n">
         <v>4</v>
       </c>
-      <c r="BM16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN16" t="inlineStr"/>
-      <c r="BO16" t="inlineStr"/>
-      <c r="BP16" t="inlineStr">
+      <c r="BO16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ16" t="inlineStr">
+      <c r="BV16" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR16" t="inlineStr">
+      <c r="BW16" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS16" t="inlineStr">
+      <c r="BX16" t="inlineStr">
         <is>
           <t>registry-compatible task=object_detection training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT16" t="inlineStr"/>
-      <c r="BU16" t="inlineStr"/>
-      <c r="BV16" t="inlineStr"/>
-      <c r="BW16" t="inlineStr">
-        <is>
-          <t>object-detection</t>
-        </is>
-      </c>
-      <c r="BX16" t="inlineStr"/>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
       <c r="CA16" t="inlineStr"/>
-      <c r="CB16" t="inlineStr"/>
+      <c r="CB16" t="inlineStr">
+        <is>
+          <t>object-detection</t>
+        </is>
+      </c>
       <c r="CC16" t="inlineStr"/>
       <c r="CD16" t="inlineStr"/>
       <c r="CE16" t="inlineStr"/>
@@ -4749,7 +4994,12 @@
       <c r="CI16" t="inlineStr"/>
       <c r="CJ16" t="inlineStr"/>
       <c r="CK16" t="inlineStr"/>
-      <c r="CL16" t="inlineStr">
+      <c r="CL16" t="inlineStr"/>
+      <c r="CM16" t="inlineStr"/>
+      <c r="CN16" t="inlineStr"/>
+      <c r="CO16" t="inlineStr"/>
+      <c r="CP16" t="inlineStr"/>
+      <c r="CQ16" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "german_traffic_sign_detection", "dataset_variant": 0, "knob_variant": 0, "model_family": "yolos", "model_registry_key": "yolos-small_objdet", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -4853,7 +5103,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -4946,50 +5196,60 @@
       <c r="BJ17" t="b">
         <v>1</v>
       </c>
-      <c r="BK17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL17" t="n">
+      <c r="BK17" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL17" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN17" t="n">
         <v>4</v>
       </c>
-      <c r="BM17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN17" t="inlineStr"/>
-      <c r="BO17" t="inlineStr"/>
-      <c r="BP17" t="inlineStr">
+      <c r="BO17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ17" t="inlineStr">
+      <c r="BV17" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR17" t="inlineStr">
+      <c r="BW17" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS17" t="inlineStr">
+      <c r="BX17" t="inlineStr">
         <is>
           <t>registry-compatible task=image_segmentation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT17" t="inlineStr"/>
-      <c r="BU17" t="inlineStr"/>
-      <c r="BV17" t="inlineStr"/>
-      <c r="BW17" t="inlineStr">
-        <is>
-          <t>image-segmentation</t>
-        </is>
-      </c>
-      <c r="BX17" t="inlineStr"/>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
       <c r="CA17" t="inlineStr"/>
-      <c r="CB17" t="inlineStr"/>
+      <c r="CB17" t="inlineStr">
+        <is>
+          <t>image-segmentation</t>
+        </is>
+      </c>
       <c r="CC17" t="inlineStr"/>
       <c r="CD17" t="inlineStr"/>
       <c r="CE17" t="inlineStr"/>
@@ -4999,7 +5259,12 @@
       <c r="CI17" t="inlineStr"/>
       <c r="CJ17" t="inlineStr"/>
       <c r="CK17" t="inlineStr"/>
-      <c r="CL17" t="inlineStr">
+      <c r="CL17" t="inlineStr"/>
+      <c r="CM17" t="inlineStr"/>
+      <c r="CN17" t="inlineStr"/>
+      <c r="CO17" t="inlineStr"/>
+      <c r="CP17" t="inlineStr"/>
+      <c r="CQ17" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "ade20k_mini_segmentation", "dataset_variant": 0, "knob_variant": 0, "model_family": "segformer", "model_registry_key": "segformer-b1_seg", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -5103,7 +5368,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 2e-05, "max_samples": 96, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -5196,50 +5461,60 @@
       <c r="BJ18" t="b">
         <v>1</v>
       </c>
-      <c r="BK18" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL18" t="n">
+      <c r="BK18" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL18" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN18" t="n">
         <v>4</v>
       </c>
-      <c r="BM18" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN18" t="inlineStr"/>
-      <c r="BO18" t="inlineStr"/>
-      <c r="BP18" t="inlineStr">
+      <c r="BO18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP18" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR18" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ18" t="inlineStr">
+      <c r="BV18" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR18" t="inlineStr">
+      <c r="BW18" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS18" t="inlineStr">
+      <c r="BX18" t="inlineStr">
         <is>
           <t>registry-compatible task=image_segmentation training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT18" t="inlineStr"/>
-      <c r="BU18" t="inlineStr"/>
-      <c r="BV18" t="inlineStr"/>
-      <c r="BW18" t="inlineStr">
-        <is>
-          <t>image-segmentation</t>
-        </is>
-      </c>
-      <c r="BX18" t="inlineStr"/>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
       <c r="CA18" t="inlineStr"/>
-      <c r="CB18" t="inlineStr"/>
+      <c r="CB18" t="inlineStr">
+        <is>
+          <t>image-segmentation</t>
+        </is>
+      </c>
       <c r="CC18" t="inlineStr"/>
       <c r="CD18" t="inlineStr"/>
       <c r="CE18" t="inlineStr"/>
@@ -5249,7 +5524,12 @@
       <c r="CI18" t="inlineStr"/>
       <c r="CJ18" t="inlineStr"/>
       <c r="CK18" t="inlineStr"/>
-      <c r="CL18" t="inlineStr">
+      <c r="CL18" t="inlineStr"/>
+      <c r="CM18" t="inlineStr"/>
+      <c r="CN18" t="inlineStr"/>
+      <c r="CO18" t="inlineStr"/>
+      <c r="CP18" t="inlineStr"/>
+      <c r="CQ18" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "hot_building_segmentation", "dataset_variant": 0, "knob_variant": 0, "model_family": "segformer", "model_registry_key": "segformer-b4_seg", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -5357,7 +5637,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 64, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 8, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 64, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 2, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -5452,50 +5732,60 @@
       <c r="BJ19" t="b">
         <v>1</v>
       </c>
-      <c r="BK19" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL19" t="n">
+      <c r="BK19" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL19" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN19" t="n">
         <v>4</v>
       </c>
-      <c r="BM19" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN19" t="inlineStr"/>
-      <c r="BO19" t="inlineStr"/>
-      <c r="BP19" t="inlineStr">
+      <c r="BO19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR19" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ19" t="inlineStr">
+      <c r="BV19" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR19" t="inlineStr">
+      <c r="BW19" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS19" t="inlineStr">
+      <c r="BX19" t="inlineStr">
         <is>
           <t>registry-compatible task=image_captioning training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT19" t="inlineStr"/>
-      <c r="BU19" t="inlineStr"/>
-      <c r="BV19" t="inlineStr"/>
-      <c r="BW19" t="inlineStr">
-        <is>
-          <t>image-to-text</t>
-        </is>
-      </c>
-      <c r="BX19" t="inlineStr"/>
       <c r="BY19" t="inlineStr"/>
       <c r="BZ19" t="inlineStr"/>
       <c r="CA19" t="inlineStr"/>
-      <c r="CB19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr">
+        <is>
+          <t>image-to-text</t>
+        </is>
+      </c>
       <c r="CC19" t="inlineStr"/>
       <c r="CD19" t="inlineStr"/>
       <c r="CE19" t="inlineStr"/>
@@ -5505,7 +5795,12 @@
       <c r="CI19" t="inlineStr"/>
       <c r="CJ19" t="inlineStr"/>
       <c r="CK19" t="inlineStr"/>
-      <c r="CL19" t="inlineStr">
+      <c r="CL19" t="inlineStr"/>
+      <c r="CM19" t="inlineStr"/>
+      <c r="CN19" t="inlineStr"/>
+      <c r="CO19" t="inlineStr"/>
+      <c r="CP19" t="inlineStr"/>
+      <c r="CQ19" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "flickr8k_captioning", "dataset_variant": 0, "knob_variant": 0, "model_family": "git", "model_registry_key": "git-base-coco-caption", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -5613,7 +5908,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "learning_rate": 0.0001, "max_length": 48, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 16, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.0001, "max_length": 48, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -5716,50 +6011,60 @@
       <c r="BJ20" t="b">
         <v>1</v>
       </c>
-      <c r="BK20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL20" t="n">
+      <c r="BK20" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL20" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN20" t="n">
         <v>4</v>
       </c>
-      <c r="BM20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN20" t="inlineStr"/>
-      <c r="BO20" t="inlineStr"/>
-      <c r="BP20" t="inlineStr">
+      <c r="BO20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR20" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr">
         <is>
           <t>hf_registry</t>
         </is>
       </c>
-      <c r="BQ20" t="inlineStr">
+      <c r="BV20" t="inlineStr">
         <is>
           <t>task_head</t>
         </is>
       </c>
-      <c r="BR20" t="inlineStr">
+      <c r="BW20" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS20" t="inlineStr">
+      <c r="BX20" t="inlineStr">
         <is>
           <t>registry-compatible task=visual_question_answering training_regime=finetune_transfer</t>
         </is>
       </c>
-      <c r="BT20" t="inlineStr"/>
-      <c r="BU20" t="inlineStr"/>
-      <c r="BV20" t="inlineStr"/>
-      <c r="BW20" t="inlineStr">
-        <is>
-          <t>visual-question-answering</t>
-        </is>
-      </c>
-      <c r="BX20" t="inlineStr"/>
       <c r="BY20" t="inlineStr"/>
       <c r="BZ20" t="inlineStr"/>
       <c r="CA20" t="inlineStr"/>
-      <c r="CB20" t="inlineStr"/>
+      <c r="CB20" t="inlineStr">
+        <is>
+          <t>visual-question-answering</t>
+        </is>
+      </c>
       <c r="CC20" t="inlineStr"/>
       <c r="CD20" t="inlineStr"/>
       <c r="CE20" t="inlineStr"/>
@@ -5769,7 +6074,12 @@
       <c r="CI20" t="inlineStr"/>
       <c r="CJ20" t="inlineStr"/>
       <c r="CK20" t="inlineStr"/>
-      <c r="CL20" t="inlineStr">
+      <c r="CL20" t="inlineStr"/>
+      <c r="CM20" t="inlineStr"/>
+      <c r="CN20" t="inlineStr"/>
+      <c r="CO20" t="inlineStr"/>
+      <c r="CP20" t="inlineStr"/>
+      <c r="CQ20" t="inlineStr">
         <is>
           <t>{"dataset_registry_key": "vqav2", "dataset_variant": 0, "knob_variant": 0, "model_family": "blip", "model_registry_key": "blip-vqa-base", "split_variant": 0, "training_regime": "finetune_transfer"}</t>
         </is>
@@ -5853,7 +6163,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
@@ -5934,42 +6244,52 @@
       <c r="BJ21" t="b">
         <v>1</v>
       </c>
-      <c r="BK21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL21" t="n">
+      <c r="BK21" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL21" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN21" t="n">
         <v>4</v>
       </c>
-      <c r="BM21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN21" t="inlineStr"/>
-      <c r="BO21" t="inlineStr"/>
-      <c r="BP21" t="inlineStr">
+      <c r="BO21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr">
         <is>
           <t>generic_registry</t>
         </is>
       </c>
-      <c r="BQ21" t="inlineStr">
+      <c r="BV21" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="BR21" t="inlineStr">
+      <c r="BW21" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS21" t="inlineStr">
+      <c r="BX21" t="inlineStr">
         <is>
           <t>generic manifest-compatible task runner</t>
         </is>
       </c>
-      <c r="BT21" t="inlineStr"/>
-      <c r="BU21" t="inlineStr"/>
-      <c r="BV21" t="inlineStr"/>
-      <c r="BW21" t="inlineStr"/>
-      <c r="BX21" t="inlineStr"/>
       <c r="BY21" t="inlineStr"/>
       <c r="BZ21" t="inlineStr"/>
       <c r="CA21" t="inlineStr"/>
@@ -5984,6 +6304,11 @@
       <c r="CJ21" t="inlineStr"/>
       <c r="CK21" t="inlineStr"/>
       <c r="CL21" t="inlineStr"/>
+      <c r="CM21" t="inlineStr"/>
+      <c r="CN21" t="inlineStr"/>
+      <c r="CO21" t="inlineStr"/>
+      <c r="CP21" t="inlineStr"/>
+      <c r="CQ21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6063,7 +6388,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>{"batch_size": 64, "device": "auto", "distribution_type": "iid", "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 64, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -6144,42 +6469,52 @@
       <c r="BJ22" t="b">
         <v>1</v>
       </c>
-      <c r="BK22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL22" t="n">
+      <c r="BK22" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL22" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN22" t="n">
         <v>4</v>
       </c>
-      <c r="BM22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN22" t="inlineStr"/>
-      <c r="BO22" t="inlineStr"/>
-      <c r="BP22" t="inlineStr">
+      <c r="BO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP22" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR22" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr">
         <is>
           <t>generic_registry</t>
         </is>
       </c>
-      <c r="BQ22" t="inlineStr">
+      <c r="BV22" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="BR22" t="inlineStr">
+      <c r="BW22" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS22" t="inlineStr">
+      <c r="BX22" t="inlineStr">
         <is>
           <t>generic manifest-compatible task runner</t>
         </is>
       </c>
-      <c r="BT22" t="inlineStr"/>
-      <c r="BU22" t="inlineStr"/>
-      <c r="BV22" t="inlineStr"/>
-      <c r="BW22" t="inlineStr"/>
-      <c r="BX22" t="inlineStr"/>
       <c r="BY22" t="inlineStr"/>
       <c r="BZ22" t="inlineStr"/>
       <c r="CA22" t="inlineStr"/>
@@ -6194,6 +6529,11 @@
       <c r="CJ22" t="inlineStr"/>
       <c r="CK22" t="inlineStr"/>
       <c r="CL22" t="inlineStr"/>
+      <c r="CM22" t="inlineStr"/>
+      <c r="CN22" t="inlineStr"/>
+      <c r="CO22" t="inlineStr"/>
+      <c r="CP22" t="inlineStr"/>
+      <c r="CQ22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6273,7 +6613,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "adam", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
@@ -6354,42 +6694,52 @@
       <c r="BJ23" t="b">
         <v>1</v>
       </c>
-      <c r="BK23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL23" t="n">
+      <c r="BK23" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL23" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN23" t="n">
         <v>4</v>
       </c>
-      <c r="BM23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN23" t="inlineStr"/>
-      <c r="BO23" t="inlineStr"/>
-      <c r="BP23" t="inlineStr">
+      <c r="BO23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR23" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr">
         <is>
           <t>generic_registry</t>
         </is>
       </c>
-      <c r="BQ23" t="inlineStr">
+      <c r="BV23" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="BR23" t="inlineStr">
+      <c r="BW23" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS23" t="inlineStr">
+      <c r="BX23" t="inlineStr">
         <is>
           <t>generic manifest-compatible task runner</t>
         </is>
       </c>
-      <c r="BT23" t="inlineStr"/>
-      <c r="BU23" t="inlineStr"/>
-      <c r="BV23" t="inlineStr"/>
-      <c r="BW23" t="inlineStr"/>
-      <c r="BX23" t="inlineStr"/>
       <c r="BY23" t="inlineStr"/>
       <c r="BZ23" t="inlineStr"/>
       <c r="CA23" t="inlineStr"/>
@@ -6404,6 +6754,11 @@
       <c r="CJ23" t="inlineStr"/>
       <c r="CK23" t="inlineStr"/>
       <c r="CL23" t="inlineStr"/>
+      <c r="CM23" t="inlineStr"/>
+      <c r="CN23" t="inlineStr"/>
+      <c r="CO23" t="inlineStr"/>
+      <c r="CP23" t="inlineStr"/>
+      <c r="CQ23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6483,7 +6838,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 32, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 3, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -6564,42 +6919,52 @@
       <c r="BJ24" t="b">
         <v>1</v>
       </c>
-      <c r="BK24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL24" t="n">
+      <c r="BK24" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL24" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN24" t="n">
         <v>4</v>
       </c>
-      <c r="BM24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN24" t="inlineStr"/>
-      <c r="BO24" t="inlineStr"/>
-      <c r="BP24" t="inlineStr">
+      <c r="BO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr">
         <is>
           <t>generic_registry</t>
         </is>
       </c>
-      <c r="BQ24" t="inlineStr">
+      <c r="BV24" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="BR24" t="inlineStr">
+      <c r="BW24" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS24" t="inlineStr">
+      <c r="BX24" t="inlineStr">
         <is>
           <t>generic manifest-compatible task runner</t>
         </is>
       </c>
-      <c r="BT24" t="inlineStr"/>
-      <c r="BU24" t="inlineStr"/>
-      <c r="BV24" t="inlineStr"/>
-      <c r="BW24" t="inlineStr"/>
-      <c r="BX24" t="inlineStr"/>
       <c r="BY24" t="inlineStr"/>
       <c r="BZ24" t="inlineStr"/>
       <c r="CA24" t="inlineStr"/>
@@ -6614,6 +6979,11 @@
       <c r="CJ24" t="inlineStr"/>
       <c r="CK24" t="inlineStr"/>
       <c r="CL24" t="inlineStr"/>
+      <c r="CM24" t="inlineStr"/>
+      <c r="CN24" t="inlineStr"/>
+      <c r="CO24" t="inlineStr"/>
+      <c r="CP24" t="inlineStr"/>
+      <c r="CQ24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6693,7 +7063,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>{"batch_size": 64, "device": "auto", "distribution_type": "iid", "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
+          <t>{"batch_size": 64, "device": "auto", "distribution_type": "iid", "enable_perturbation_metrics": true, "learning_rate": 0.001, "max_samples": 128, "mixed_precision": false, "momentum": 0.0, "optimizer": "none", "perturbation_sample_count": 1, "save_weights": false, "split_strategy": "iid", "timeout_s": 3600, "training_epochs": 1, "weight_decay": 0.0}</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
@@ -6774,42 +7144,52 @@
       <c r="BJ25" t="b">
         <v>1</v>
       </c>
-      <c r="BK25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BL25" t="n">
+      <c r="BK25" t="b">
+        <v>1</v>
+      </c>
+      <c r="BL25" t="b">
+        <v>0</v>
+      </c>
+      <c r="BM25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BN25" t="n">
         <v>4</v>
       </c>
-      <c r="BM25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BN25" t="inlineStr"/>
-      <c r="BO25" t="inlineStr"/>
-      <c r="BP25" t="inlineStr">
+      <c r="BO25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP25" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR25" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr">
         <is>
           <t>generic_registry</t>
         </is>
       </c>
-      <c r="BQ25" t="inlineStr">
+      <c r="BV25" t="inlineStr">
         <is>
           <t>service</t>
         </is>
       </c>
-      <c r="BR25" t="inlineStr">
+      <c r="BW25" t="inlineStr">
         <is>
           <t>compatible</t>
         </is>
       </c>
-      <c r="BS25" t="inlineStr">
+      <c r="BX25" t="inlineStr">
         <is>
           <t>generic manifest-compatible task runner</t>
         </is>
       </c>
-      <c r="BT25" t="inlineStr"/>
-      <c r="BU25" t="inlineStr"/>
-      <c r="BV25" t="inlineStr"/>
-      <c r="BW25" t="inlineStr"/>
-      <c r="BX25" t="inlineStr"/>
       <c r="BY25" t="inlineStr"/>
       <c r="BZ25" t="inlineStr"/>
       <c r="CA25" t="inlineStr"/>
@@ -6824,6 +7204,11 @@
       <c r="CJ25" t="inlineStr"/>
       <c r="CK25" t="inlineStr"/>
       <c r="CL25" t="inlineStr"/>
+      <c r="CM25" t="inlineStr"/>
+      <c r="CN25" t="inlineStr"/>
+      <c r="CO25" t="inlineStr"/>
+      <c r="CP25" t="inlineStr"/>
+      <c r="CQ25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>